<commit_message>
feat: optimize dictionary to distinguish business-specific intents
- Refined dictionary mappings to differentiate shared filter intents across distinct banking use cases
- Improved contextual handling to ensure outputs align with domain-specific requirements
- Enhanced rule engine accuracy by tailoring examples to relevant business scenarios
</commit_message>
<xml_diff>
--- a/Text2SQL_Template/output/generated_datasets/ddq_autogen_customer.xlsx
+++ b/Text2SQL_Template/output/generated_datasets/ddq_autogen_customer.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="64">
   <si>
     <t>document</t>
   </si>
@@ -31,113 +31,118 @@
     <t>metadata</t>
   </si>
   <si>
-    <t xml:space="preserve">customer | Tra cứu </t>
+    <t>customer | Tra cứu primary key</t>
   </si>
   <si>
     <t>customer | Tra cứu mã khách hàng</t>
   </si>
   <si>
-    <t>customer | Tra cứu mã số khách hàng</t>
+    <t>customer | Tra cứu số khách hàng</t>
   </si>
   <si>
     <t>customer | Tra cứu chi nhánh mã khách hàng</t>
   </si>
   <si>
-    <t>customer | Lọc theo mã khách hàng</t>
-  </si>
-  <si>
-    <t>customer | Lọc theo khách hàng</t>
-  </si>
-  <si>
-    <t>customer | Lọc thời gian</t>
+    <t>customer | Lọc theo loại mã khách hàng</t>
+  </si>
+  <si>
+    <t>customer | Lọc theo trạng thái khách hàng</t>
+  </si>
+  <si>
+    <t>customer | Lọc thời gian theo init date</t>
   </si>
   <si>
     <t>customer | Thống kê phí</t>
   </si>
   <si>
-    <t xml:space="preserve">customer | Lọc theo </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tìm kiếm chính xác theo </t>
+    <t>customer | Lọc theo trạng thái bản ghi</t>
+  </si>
+  <si>
+    <t>customer | Lọc thời gian theo ngày tháng năm sinh.</t>
+  </si>
+  <si>
+    <t>Tìm kiếm chính xác theo primary key</t>
   </si>
   <si>
     <t>Tìm kiếm chính xác theo mã khách hàng</t>
   </si>
   <si>
-    <t>Tìm kiếm chính xác theo mã số khách hàng</t>
+    <t>Tìm kiếm chính xác theo số khách hàng</t>
   </si>
   <si>
     <t>Tìm kiếm chính xác theo chi nhánh mã khách hàng</t>
   </si>
   <si>
-    <t>Phân nhóm giao dịch theo mã khách hàng</t>
-  </si>
-  <si>
-    <t>Phân nhóm giao dịch theo khách hàng</t>
-  </si>
-  <si>
-    <t>Truy vấn lịch sử theo thời gian cụ thể</t>
+    <t>Phân nhóm giao dịch theo loại mã khách hàng</t>
+  </si>
+  <si>
+    <t>Phân nhóm giao dịch theo trạng thái khách hàng</t>
+  </si>
+  <si>
+    <t>Truy vấn lịch sử dựa trên cột init date</t>
   </si>
   <si>
     <t>Tính tổng giá trị phí</t>
   </si>
   <si>
-    <t xml:space="preserve">Phân nhóm giao dịch theo </t>
-  </si>
-  <si>
-    <t>Check giao dịch 865
-Kiểm tra lệnh 865 đang ở trạng thái nào
-Tra cứu khách hàng 865 tuần này
-Xem chi tiết khách hàng số 865</t>
-  </si>
-  <si>
-    <t>Sao kê cho mã khách hàng 8062062
-Liệt kê giao dịch của khách hàng 8062062
-Xem lịch sử của mã khách hàng 8062062</t>
-  </si>
-  <si>
-    <t>Sao kê cho mã khách hàng 3647072
-Liệt kê giao dịch của khách hàng 3647072
-Xem lịch sử của mã khách hàng 3647072</t>
-  </si>
-  <si>
-    <t>Liệt kê giao dịch của khách hàng 2252118
-Xem lịch sử của mã số khách hàng 2252118
-Sao kê cho mã số khách hàng 2252118</t>
-  </si>
-  <si>
-    <t>Xem lịch sử của chi nhánh mã khách hàng TYPE_VK80
-Sao kê cho chi nhánh mã khách hàng TYPE_VK80
-Liệt kê giao dịch của khách hàng TYPE_VK80</t>
-  </si>
-  <si>
-    <t>danh sách khách hàng hóa đơn điện
-khách hàng hóa đơn điện
-lọc các khách hàng đang hóa đơn điện
-khách hàng napas 247
-khách hàng thanh toán qr
-danh sách khách hàng napas 247
-danh sách khách hàng thanh toán qr
-lọc các khách hàng đang napas 247
-lọc các khách hàng đang thanh toán qr</t>
-  </si>
-  <si>
-    <t>khách hàng bị treo
-danh sách khách hàng hoàn tất
+    <t>Phân nhóm giao dịch theo trạng thái bản ghi</t>
+  </si>
+  <si>
+    <t>Truy vấn lịch sử dựa trên cột ngày tháng năm sinh.</t>
+  </si>
+  <si>
+    <t>Kiểm tra lệnh 569 xem thành công chưa
+Check giao dịch 569
+Tra cứu khách hàng 569 hôm qua
+Xem chi tiết khách hàng số 569</t>
+  </si>
+  <si>
+    <t>Liệt kê giao dịch của khách hàng 4781402
+Xem lịch sử của mã khách hàng 4781402
+Sao kê cho mã khách hàng 4781402</t>
+  </si>
+  <si>
+    <t>Sao kê cho mã khách hàng 8831657
+Xem lịch sử của mã khách hàng 8831657
+Liệt kê giao dịch của khách hàng 8831657</t>
+  </si>
+  <si>
+    <t>Sao kê cho số khách hàng 3226610
+Xem lịch sử của số khách hàng 3226610
+Liệt kê giao dịch của khách hàng 3226610</t>
+  </si>
+  <si>
+    <t>Xem lịch sử của chi nhánh mã khách hàng CAT_5W39
+Liệt kê giao dịch của khách hàng CAT_5W39
+Sao kê cho chi nhánh mã khách hàng CAT_5W39</t>
+  </si>
+  <si>
+    <t>lọc các khách hàng đang chuyển liên ngân hàng
+lọc các khách hàng đang chuyển nội bộ
+danh sách khách hàng chuyển liên ngân hàng
+khách hàng chuyển nhanh
+khách hàng chuyển liên ngân hàng
+khách hàng chuyển nội bộ
+danh sách khách hàng chuyển nhanh
+lọc các khách hàng đang chuyển nhanh
+danh sách khách hàng chuyển nội bộ</t>
+  </si>
+  <si>
+    <t>lọc các khách hàng đang bị treo
+lọc các khách hàng đang đã xong
 danh sách khách hàng bị treo
-khách hàng hoàn tất
+khách hàng đã xong
+khách hàng treo
+danh sách khách hàng đã xong
+khách hàng bị treo
 danh sách khách hàng treo
-lọc các khách hàng đang treo
-lọc các khách hàng đang hoàn tất
-khách hàng treo
-lọc các khách hàng đang bị treo</t>
-  </si>
-  <si>
-    <t>Sao kê khách hàng từ ngày 2026-01-15 đến ngày 2026-01-29
-Lịch sử khách hàng trong khoảng 2026-01-15 - 2026-01-29
-Xem khách hàng từ 2026-01-15 tới 2026-01-29
-Tra soát giao dịch ngày 2026-01-15
-Xem khách hàng 30 ngày gần đây</t>
+lọc các khách hàng đang treo</t>
+  </si>
+  <si>
+    <t>Sao kê khách hàng theo init date từ ngày 2025-12-13 đến ngày 2026-01-29
+Lọc khách hàng có init date trong khoảng 2025-12-13 - 2026-01-29
+Xem lịch sử khách hàng dựa trên init date từ 2025-12-13 tới 2026-01-29
+Kiểm tra các khách hàng với init date là ngày 2025-12-13</t>
   </si>
   <si>
     <t>Tổng phí là bao nhiêu?
@@ -145,47 +150,46 @@
 Thống kê phí hôm nay</t>
   </si>
   <si>
-    <t>danh sách khách hàng hoàn tất
-khách hàng hoàn tất
+    <t>lọc các khách hàng đang bị treo
+lọc các khách hàng đang quá giờ
+lọc các khách hàng đang đã xong
+danh sách khách hàng bị treo
+danh sách khách hàng quá giờ
+khách hàng đã xong
+danh sách khách hàng đã xong
+khách hàng bị treo
+khách hàng quá giờ</t>
+  </si>
+  <si>
+    <t>Sao kê khách hàng theo ngày tháng năm sinh. từ ngày 2025-12-05 đến ngày 2026-01-29
+Lọc khách hàng có ngày tháng năm sinh. trong khoảng 2025-12-05 - 2026-01-29
+Xem lịch sử khách hàng dựa trên ngày tháng năm sinh. từ 2025-12-05 tới 2026-01-29
+Kiểm tra các khách hàng với ngày tháng năm sinh. là ngày 2025-12-05</t>
+  </si>
+  <si>
+    <t>khách hàng hoàn tất
+danh sách khách hàng lỗi
+lọc các khách hàng đang lỗi
+khách hàng lỗi
+danh sách khách hàng hoàn tất
+lọc các khách hàng đang hoàn tất
+khách hàng treo
+danh sách khách hàng treo
+lọc các khách hàng đang treo</t>
+  </si>
+  <si>
+    <t>danh sách khách hàng xử lý
+danh sách khách hàng lỗi
+lọc các khách hàng đang quá giờ
+lọc các khách hàng đang lỗi
+khách hàng lỗi
 lọc các khách hàng đang xử lý
-danh sách khách hàng thất bại
-lọc các khách hàng đang hoàn tất
-lọc các khách hàng đang thất bại
-khách hàng thất bại
-danh sách khách hàng xử lý
-khách hàng xử lý</t>
-  </si>
-  <si>
-    <t>Sao kê khách hàng từ ngày 2026-01-12 đến ngày 2026-01-29
-Lịch sử khách hàng trong khoảng 2026-01-12 - 2026-01-29
-Xem khách hàng từ 2026-01-12 tới 2026-01-29
-Tra soát giao dịch ngày 2026-01-12
-Xem khách hàng 30 ngày gần đây</t>
-  </si>
-  <si>
-    <t>khách hàng bị treo
-khách hàng quá giờ
-danh sách khách hàng bị treo
-lọc các khách hàng đang xử lý
-lọc các khách hàng đang quá giờ
 danh sách khách hàng quá giờ
-danh sách khách hàng xử lý
 khách hàng xử lý
-lọc các khách hàng đang bị treo</t>
-  </si>
-  <si>
-    <t>khách hàng bị treo
-khách hàng quá giờ
-danh sách khách hàng hoàn tất
-danh sách khách hàng bị treo
-khách hàng hoàn tất
-lọc các khách hàng đang quá giờ
-lọc các khách hàng đang hoàn tất
-danh sách khách hàng quá giờ
-lọc các khách hàng đang bị treo</t>
-  </si>
-  <si>
-    <t>, primary key, mã</t>
+khách hàng quá giờ</t>
+  </si>
+  <si>
+    <t>primary key</t>
   </si>
   <si>
     <t>mã khách hàng, số cif, mã định danh khách hàng</t>
@@ -194,31 +198,34 @@
     <t>mã khách hàng, khách hàng</t>
   </si>
   <si>
-    <t>mã số khách hàng, số khách hàng, khách hàng</t>
+    <t>số khách hàng, khách hàng, mã số khách hàng</t>
   </si>
   <si>
     <t>chi nhánh mã khách hàng, mã khách hàng</t>
   </si>
   <si>
-    <t>mã khách hàng, loại mã khách hàng, loại cif</t>
-  </si>
-  <si>
-    <t>khách hàng, active, inactive, closed..., trạng thái khách hàng</t>
-  </si>
-  <si>
-    <t>thời gian, lịch sử, ngày tháng</t>
+    <t>loại mã khách hàng, mã khách hàng, loại cif</t>
+  </si>
+  <si>
+    <t>trạng thái khách hàng, khách hàng, active, inactive, closed...</t>
+  </si>
+  <si>
+    <t>thời gian, lịch sử, init date</t>
   </si>
   <si>
     <t>tổng, thống kê</t>
   </si>
   <si>
-    <t>, trạng thái, trạng thái bản ghi</t>
-  </si>
-  <si>
-    <t>khách hàng, trước khi thay đổi, trạng thái khách hàng, trạng thái cũ khách hàng</t>
-  </si>
-  <si>
-    <t>khách hàng, sau khi cập nhật, trạng thái khách hàng, trạng thái mới khách hàng</t>
+    <t>trạng thái bản ghi</t>
+  </si>
+  <si>
+    <t>thời gian, lịch sử, ngày tháng năm sinh.</t>
+  </si>
+  <si>
+    <t>trạng thái khách hàng, khách hàng, trạng thái cũ khách hàng, trước khi thay đổi</t>
+  </si>
+  <si>
+    <t>trạng thái khách hàng, khách hàng, trạng thái mới khách hàng, sau khi cập nhật</t>
   </si>
   <si>
     <t>{"raw_text": "SELECT * FROM customer WHERE id = '{{id}}'"}</t>
@@ -640,16 +647,16 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E2" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -657,16 +664,16 @@
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E3" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -674,16 +681,16 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D4" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E4" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -691,16 +698,16 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D5" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E5" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -708,16 +715,16 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E6" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -725,16 +732,16 @@
         <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C7" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D7" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E7" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -742,16 +749,16 @@
         <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C8" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E8" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -759,16 +766,16 @@
         <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C9" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D9" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E9" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -776,16 +783,16 @@
         <v>12</v>
       </c>
       <c r="B10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C10" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D10" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E10" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -793,33 +800,33 @@
         <v>13</v>
       </c>
       <c r="B11" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D11" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E11" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C12" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D12" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="E12" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -827,16 +834,16 @@
         <v>10</v>
       </c>
       <c r="B13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D13" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="E13" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -844,16 +851,16 @@
         <v>10</v>
       </c>
       <c r="B14" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C14" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D14" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="E14" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add sentence transformer to profiler stage
- Integrated sentence transformer into the profiling process
- Updated flow to: profiler → dict builder → generator
- Improved contextual representation for downstream dictionary building and example generation
</commit_message>
<xml_diff>
--- a/Text2SQL_Template/output/generated_datasets/ddq_autogen_customer.xlsx
+++ b/Text2SQL_Template/output/generated_datasets/ddq_autogen_customer.xlsx
@@ -1,21 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\proton-intern\javisAI\6804_ddq\Text2SQL_Template\output\generated_datasets\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96CD507E-DB55-4CA3-B83D-E616269BC7EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="26537" windowHeight="15943" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -37,219 +31,219 @@
     <t>metadata</t>
   </si>
   <si>
-    <t>customer | Tra cứu primary key</t>
-  </si>
-  <si>
-    <t>customer | Tra cứu số mã khách hàng</t>
+    <t>customer | Tra cứu bản ghi này</t>
   </si>
   <si>
     <t>customer | Tra cứu mã khách hàng</t>
   </si>
   <si>
-    <t>customer | Tra cứu mã số khách hàng</t>
-  </si>
-  <si>
-    <t>customer | Tra cứu chi nhánh nơi mở/quản lý mã cif này.</t>
-  </si>
-  <si>
-    <t>customer | Lọc theo loại cif</t>
-  </si>
-  <si>
-    <t>customer | Lọc theo trạng thái hiện khách hàng</t>
-  </si>
-  <si>
-    <t>customer | Lọc thời gian theo ngày khởi tạo khách hàng trên</t>
-  </si>
-  <si>
-    <t>customer | Thống kê đánh dấu khách hàng có thuộc diện mặc định thu phí hay không</t>
-  </si>
-  <si>
-    <t>customer | Lọc theo trạng thái</t>
-  </si>
-  <si>
-    <t>customer | Lọc thời gian theo ngày tháng năm sinh.</t>
-  </si>
-  <si>
-    <t>customer | Lọc theo trước khi thay đổi</t>
-  </si>
-  <si>
-    <t>customer | Lọc theo trạng thái mới khách hàng</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác theo primary key</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác theo số mã khách hàng</t>
+    <t>customer | Tra cứu id định danh khách hàng trong nội bộ</t>
+  </si>
+  <si>
+    <t>customer | Tra cứu có thể khác với cif tùy theo cấu trúc hệ thống</t>
+  </si>
+  <si>
+    <t>customer | Tra cứu mã khách hàng chi nhánh</t>
+  </si>
+  <si>
+    <t>customer | Lọc theo khách hàng ưu tiên...</t>
+  </si>
+  <si>
+    <t>customer | Lọc theo khách hàng trạng thái</t>
+  </si>
+  <si>
+    <t>customer | Lọc thời gian theo ngày khởi tạo khách hàng trên hệ thống</t>
+  </si>
+  <si>
+    <t>customer | Thống kê trạng thái phí trạng thái</t>
+  </si>
+  <si>
+    <t>customer | Lọc theo 0-hết hiệu lực</t>
+  </si>
+  <si>
+    <t>customer | Lọc thời gian theo ngày trạng thái trạng thái</t>
+  </si>
+  <si>
+    <t>customer | Lọc theo trạng thái old khách hàng</t>
+  </si>
+  <si>
+    <t>customer | Lọc theo sau khi cập nhật</t>
+  </si>
+  <si>
+    <t>Tìm kiếm chính xác theo bản ghi này</t>
   </si>
   <si>
     <t>Tìm kiếm chính xác theo mã khách hàng</t>
   </si>
   <si>
-    <t>Tìm kiếm chính xác theo mã số khách hàng</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác theo chi nhánh nơi mở/quản lý mã cif này.</t>
-  </si>
-  <si>
-    <t>Phân nhóm giao dịch theo loại cif</t>
-  </si>
-  <si>
-    <t>Phân nhóm giao dịch theo trạng thái hiện khách hàng</t>
-  </si>
-  <si>
-    <t>Truy vấn lịch sử dựa trên cột ngày khởi tạo khách hàng trên</t>
-  </si>
-  <si>
-    <t>Tính tổng giá trị đánh dấu khách hàng có thuộc diện mặc định thu phí hay không</t>
-  </si>
-  <si>
-    <t>Phân nhóm giao dịch theo trạng thái</t>
-  </si>
-  <si>
-    <t>Truy vấn lịch sử dựa trên cột ngày tháng năm sinh.</t>
-  </si>
-  <si>
-    <t>Phân nhóm giao dịch theo trước khi thay đổi</t>
-  </si>
-  <si>
-    <t>Phân nhóm giao dịch theo trạng thái mới khách hàng</t>
-  </si>
-  <si>
-    <t>Xem chi tiết khách hàng số 374
-Tra cứu khách hàng 374
-Kiểm tra lệnh 374 đang ở trạng thái nào
-Check giao dịch 374</t>
-  </si>
-  <si>
-    <t>Xem lịch sử của số mã khách hàng 2511676
-Sao kê cho số mã khách hàng 2511676
-Liệt kê giao dịch của khách hàng 2511676</t>
-  </si>
-  <si>
-    <t>Sao kê cho mã khách hàng 5025185
-Liệt kê giao dịch của khách hàng 5025185
-Xem lịch sử của mã khách hàng 5025185</t>
-  </si>
-  <si>
-    <t>Liệt kê giao dịch của khách hàng 3416983
-Xem lịch sử của mã số khách hàng 3416983
-Sao kê cho mã số khách hàng 3416983</t>
-  </si>
-  <si>
-    <t>Liệt kê giao dịch của khách hàng CAT_7Y79
-Xem lịch sử của chi nhánh nơi mở/quản lý mã cif này. CAT_7Y79
-Sao kê cho chi nhánh nơi mở/quản lý mã cif này. CAT_7Y79</t>
-  </si>
-  <si>
-    <t>lọc các khách hàng đang chuyển nội bộ
-khách hàng chuyển nội bộ
-danh sách khách hàng chuyển nội bộ
-lọc các khách hàng đang tiền nước
-danh sách khách hàng hóa đơn điện
-khách hàng hóa đơn điện
-lọc các khách hàng đang hóa đơn điện
-danh sách khách hàng tiền nước
-khách hàng tiền nước</t>
-  </si>
-  <si>
-    <t>lọc các khách hàng đang đã xong
-danh sách khách hàng đang chờ
+    <t>Tìm kiếm chính xác theo id định danh khách hàng trong nội bộ</t>
+  </si>
+  <si>
+    <t>Tìm kiếm chính xác theo có thể khác với cif tùy theo cấu trúc hệ thống</t>
+  </si>
+  <si>
+    <t>Tìm kiếm chính xác theo mã khách hàng chi nhánh</t>
+  </si>
+  <si>
+    <t>Phân nhóm giao dịch theo khách hàng ưu tiên...</t>
+  </si>
+  <si>
+    <t>Phân nhóm giao dịch theo khách hàng trạng thái</t>
+  </si>
+  <si>
+    <t>Truy vấn lịch sử dựa trên cột ngày khởi tạo khách hàng trên hệ thống</t>
+  </si>
+  <si>
+    <t>Tính tổng giá trị trạng thái phí trạng thái</t>
+  </si>
+  <si>
+    <t>Phân nhóm giao dịch theo 0-hết hiệu lực</t>
+  </si>
+  <si>
+    <t>Truy vấn lịch sử dựa trên cột ngày trạng thái trạng thái</t>
+  </si>
+  <si>
+    <t>Phân nhóm giao dịch theo trạng thái old khách hàng</t>
+  </si>
+  <si>
+    <t>Phân nhóm giao dịch theo sau khi cập nhật</t>
+  </si>
+  <si>
+    <t>Tra cứu khách hàng 537
+Kiểm tra lệnh 537 xem thành công chưa
+Xem chi tiết khách hàng số 537
+Check giao dịch 537</t>
+  </si>
+  <si>
+    <t>Sao kê cho mã khách hàng 8481943
+Liệt kê giao dịch của khách hàng 8481943
+Xem lịch sử của mã khách hàng 8481943</t>
+  </si>
+  <si>
+    <t>Xem lịch sử của id định danh khách hàng trong nội bộ 7231162
+Liệt kê giao dịch của khách hàng 7231162
+Sao kê cho id định danh khách hàng trong nội bộ 7231162</t>
+  </si>
+  <si>
+    <t>Xem lịch sử của có thể khác với cif tùy theo cấu trúc hệ thống 6784867
+Liệt kê giao dịch của khách hàng 6784867
+Sao kê cho có thể khác với cif tùy theo cấu trúc hệ thống 6784867</t>
+  </si>
+  <si>
+    <t>Xem lịch sử của mã khách hàng chi nhánh TYPE_V35G
+Sao kê cho mã khách hàng chi nhánh TYPE_V35G
+Liệt kê giao dịch của khách hàng TYPE_V35G</t>
+  </si>
+  <si>
+    <t>lọc các khách hàng đang napas 247
+lọc các khách hàng đang nạp thẻ
+khách hàng napas 247
+danh sách khách hàng chuyển liên ngân hàng
+danh sách khách hàng nạp thẻ
+khách hàng chuyển liên ngân hàng
+khách hàng nạp thẻ
+danh sách khách hàng napas 247
+lọc các khách hàng đang chuyển liên ngân hàng</t>
+  </si>
+  <si>
+    <t>khách hàng xử lý
+lọc các khách hàng đang bị treo
+khách hàng thành công
+khách hàng bị treo
+danh sách khách hàng bị treo
+danh sách khách hàng xử lý
+lọc các khách hàng đang xử lý
+danh sách khách hàng thành công
+lọc các khách hàng đang thành công</t>
+  </si>
+  <si>
+    <t>Sao kê khách hàng theo ngày khởi tạo khách hàng trên hệ thống từ ngày 2025-12-11 đến ngày 2026-02-03
+Lọc khách hàng có ngày khởi tạo khách hàng trên hệ thống trong khoảng 2025-12-11 - 2026-02-03
+Xem lịch sử khách hàng dựa trên ngày khởi tạo khách hàng trên hệ thống từ 2025-12-11 tới 2026-02-03
+Kiểm tra các khách hàng với ngày khởi tạo khách hàng trên hệ thống là ngày 2025-12-11</t>
+  </si>
+  <si>
+    <t>Tổng trạng thái phí trạng thái là bao nhiêu?
+Tính tổng trạng thái phí trạng thái của các giao dịch thành công
+Thống kê trạng thái phí trạng thái hôm nay</t>
+  </si>
+  <si>
+    <t>lọc các khách hàng đang thất bại
+lọc các khách hàng đang quá giờ
+danh sách khách hàng quá giờ
+khách hàng quá giờ
+lọc các khách hàng đang treo
+khách hàng treo
+danh sách khách hàng treo
+khách hàng thất bại
+danh sách khách hàng thất bại</t>
+  </si>
+  <si>
+    <t>Sao kê khách hàng theo ngày trạng thái trạng thái từ ngày 2025-12-14 đến ngày 2026-02-03
+Lọc khách hàng có ngày trạng thái trạng thái trong khoảng 2025-12-14 - 2026-02-03
+Xem lịch sử khách hàng dựa trên ngày trạng thái trạng thái từ 2025-12-14 tới 2026-02-03
+Kiểm tra các khách hàng với ngày trạng thái trạng thái là ngày 2025-12-14</t>
+  </si>
+  <si>
+    <t>lọc các khách hàng đang thất bại
+khách hàng xử lý
+khách hàng thành công
+danh sách khách hàng xử lý
+lọc các khách hàng đang xử lý
+danh sách khách hàng thành công
+khách hàng thất bại
+danh sách khách hàng thất bại
+lọc các khách hàng đang thành công</t>
+  </si>
+  <si>
+    <t>lọc các khách hàng đang quá giờ
+khách hàng xử lý
+danh sách khách hàng quá giờ
+danh sách khách hàng xử lý
+lọc các khách hàng đang xử lý
+khách hàng quá giờ
 lọc các khách hàng đang lỗi
-khách hàng đang chờ
-lọc các khách hàng đang đang chờ
-danh sách khách hàng lỗi
 khách hàng lỗi
-khách hàng đã xong
-danh sách khách hàng đã xong</t>
-  </si>
-  <si>
-    <t>Sao kê khách hàng theo ngày khởi tạo khách hàng trên từ ngày 2025-12-18 đến ngày 2026-02-03
-Lọc khách hàng có ngày khởi tạo khách hàng trên trong khoảng 2025-12-18 - 2026-02-03
-Xem lịch sử khách hàng dựa trên ngày khởi tạo khách hàng trên từ 2025-12-18 tới 2026-02-03
-Kiểm tra các khách hàng với ngày khởi tạo khách hàng trên là ngày 2025-12-18</t>
-  </si>
-  <si>
-    <t>Tổng đánh dấu khách hàng có thuộc diện mặc định thu phí hay không là bao nhiêu?
-Tính tổng đánh dấu khách hàng có thuộc diện mặc định thu phí hay không của các giao dịch thành công
-Thống kê đánh dấu khách hàng có thuộc diện mặc định thu phí hay không hôm nay</t>
-  </si>
-  <si>
-    <t>danh sách khách hàng treo
-lọc các khách hàng đang thành công
-khách hàng bị treo
-lọc các khách hàng đang bị treo
-lọc các khách hàng đang treo
-danh sách khách hàng thành công
-danh sách khách hàng bị treo
-khách hàng thành công
-khách hàng treo</t>
-  </si>
-  <si>
-    <t>Sao kê khách hàng theo ngày tháng năm sinh. từ ngày 2025-12-15 đến ngày 2026-02-03
-Lọc khách hàng có ngày tháng năm sinh. trong khoảng 2025-12-15 - 2026-02-03
-Xem lịch sử khách hàng dựa trên ngày tháng năm sinh. từ 2025-12-15 tới 2026-02-03
-Kiểm tra các khách hàng với ngày tháng năm sinh. là ngày 2025-12-15</t>
-  </si>
-  <si>
-    <t>khách hàng xử lý
-lọc các khách hàng đang thành công
-khách hàng bị treo
-lọc các khách hàng đang bị treo
-danh sách khách hàng thành công
-danh sách khách hàng xử lý
-danh sách khách hàng bị treo
-khách hàng thành công
-lọc các khách hàng đang xử lý</t>
-  </si>
-  <si>
-    <t>danh sách khách hàng đang chờ
-lọc các khách hàng đang hết hạn
-danh sách khách hàng hết hạn
-khách hàng hết hạn
-lọc các khách hàng đang lỗi
-khách hàng đang chờ
-lọc các khách hàng đang đang chờ
-danh sách khách hàng lỗi
-khách hàng lỗi</t>
-  </si>
-  <si>
-    <t>primary key, số, mã, id tự tăng, khóa chính, id tự tăng là khóa chính bản ghi này</t>
-  </si>
-  <si>
-    <t>số mã khách hàng, mã khách hàng, customer information file, số cif mã định danh duy nhất khách hàng ngân hàng, mã định danh khách hàng, số cif, số số khách hàng</t>
-  </si>
-  <si>
-    <t>mã khách hàng, id định danh khách hàng nội bộ., số khách hàng, id định danh khách hàng trong nội bộ</t>
-  </si>
-  <si>
-    <t>mã số khách hàng, số khách hàng, có thể khác với cif tùy theo cấu trúc hệ thống</t>
-  </si>
-  <si>
-    <t>chi nhánh nơi mở/quản lý mã cif này., chi nhánh nơi mở/quản lý mã cif này, số khách hàng chi nhánh, mã khách hàng chi nhánh</t>
-  </si>
-  <si>
-    <t>loại cif, loại mã khách hàng, loại số khách hàng, ví dụ: cá nhân, doanh nghiệp, khách hàng ưu tiên...</t>
-  </si>
-  <si>
-    <t>trạng thái hiện khách hàng, active, inactive, closed..., trạng thái hiện tại khách hàng, trạng thái khách hàng</t>
-  </si>
-  <si>
-    <t>thời gian, lịch sử, ngày khởi tạo khách hàng trên</t>
+danh sách khách hàng lỗi</t>
+  </si>
+  <si>
+    <t>bản ghi này, mã, primary key, số, id tự tăng là khóa chính bản ghi này</t>
+  </si>
+  <si>
+    <t>mã khách hàng, số số khách hàng, số cif, số cif mã định danh duy nhất khách hàng ngân hàng, số mã khách hàng, customer information file, mã định danh khách hàng, số khách hàng</t>
+  </si>
+  <si>
+    <t>id định danh khách hàng trong nội bộ, mã khách hàng, số khách hàng, định danh khách hàng nội bộ</t>
+  </si>
+  <si>
+    <t>có thể khác với cif tùy theo cấu trúc hệ thống, số khách hàng, mã số khách hàng</t>
+  </si>
+  <si>
+    <t>mã khách hàng chi nhánh, chi nhánh nơi mở, quản lý mã cif này, số khách hàng chi nhánh, khách hàng chi nhánh, chi nhánh nơi mở/quản lý mã cif này</t>
+  </si>
+  <si>
+    <t>khách hàng ưu tiên..., loại mã khách hàng, cá nhân, loại số khách hàng, doanh nghiệp, loại khách hàng, loại cif</t>
+  </si>
+  <si>
+    <t>khách hàng trạng thái, inactive, closed..., active, trạng thái hiện khách hàng, trạng thái khách hàng</t>
+  </si>
+  <si>
+    <t>thời gian, lịch sử, ngày khởi tạo khách hàng trên hệ thống</t>
   </si>
   <si>
     <t>tổng, thống kê</t>
   </si>
   <si>
-    <t>trạng thái, ví dụ: 1-hiệu lực, 0-hết hiệu lực, trạng thái bản ghi</t>
-  </si>
-  <si>
-    <t>thời gian, lịch sử, ngày tháng năm sinh.</t>
-  </si>
-  <si>
-    <t>trước khi thay đổi, trạng thái old khách hàng, trạng thái cũ khách hàng</t>
-  </si>
-  <si>
-    <t>trạng thái mới khách hàng, sau khi cập nhật, trạng thái new khách hàng</t>
+    <t>0-hết hiệu lực, trạng thái bản ghi, 1-hiệu lực, trạng thái</t>
+  </si>
+  <si>
+    <t>thời gian, lịch sử, ngày trạng thái trạng thái</t>
+  </si>
+  <si>
+    <t>trạng thái old khách hàng, trạng thái cũ khách hàng, trước khi thay đổi, người thụ hưởng khách hàng trạng thái</t>
+  </si>
+  <si>
+    <t>sau khi cập nhật, trạng thái mới khách hàng, nội dung khách hàng trạng thái, trạng thái new khách hàng</t>
   </si>
   <si>
     <t>{"raw_text": "SELECT * FROM customer WHERE id = '{{id}}'"}</t>
@@ -294,8 +288,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -347,13 +341,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -361,21 +352,13 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -413,7 +396,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -447,7 +430,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -482,10 +464,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -658,14 +639,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E14"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
-  <cols>
-    <col min="1" max="5" width="41.921875" style="2" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -682,224 +660,224 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="58.3" x14ac:dyDescent="0.4">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" t="s">
         <v>31</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" t="s">
         <v>44</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="58.3" x14ac:dyDescent="0.4">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" t="s">
         <v>32</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" t="s">
         <v>45</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="43.75" x14ac:dyDescent="0.4">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" t="s">
         <v>33</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" t="s">
         <v>46</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="43.75" x14ac:dyDescent="0.4">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" t="s">
         <v>34</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" t="s">
         <v>47</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="72.900000000000006" x14ac:dyDescent="0.4">
-      <c r="A6" s="2" t="s">
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" t="s">
         <v>35</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" t="s">
         <v>48</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="131.15" x14ac:dyDescent="0.4">
-      <c r="A7" s="2" t="s">
+    <row r="7" spans="1:5">
+      <c r="A7" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" t="s">
         <v>23</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" t="s">
         <v>36</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" t="s">
         <v>49</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="131.15" x14ac:dyDescent="0.4">
-      <c r="A8" s="2" t="s">
+    <row r="8" spans="1:5">
+      <c r="A8" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" t="s">
         <v>24</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" t="s">
         <v>37</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" t="s">
         <v>50</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="131.15" x14ac:dyDescent="0.4">
-      <c r="A9" s="2" t="s">
+    <row r="9" spans="1:5">
+      <c r="A9" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" t="s">
         <v>38</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" t="s">
         <v>51</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="102" x14ac:dyDescent="0.4">
-      <c r="A10" s="2" t="s">
+    <row r="10" spans="1:5">
+      <c r="A10" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" t="s">
         <v>39</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" t="s">
         <v>52</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E10" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="131.15" x14ac:dyDescent="0.4">
-      <c r="A11" s="2" t="s">
+    <row r="11" spans="1:5">
+      <c r="A11" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" t="s">
         <v>40</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" t="s">
         <v>53</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="E11" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="116.6" x14ac:dyDescent="0.4">
-      <c r="A12" s="2" t="s">
+    <row r="12" spans="1:5">
+      <c r="A12" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" t="s">
         <v>28</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" t="s">
         <v>41</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D12" t="s">
         <v>54</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="E12" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="131.15" x14ac:dyDescent="0.4">
-      <c r="A13" s="2" t="s">
+    <row r="13" spans="1:5">
+      <c r="A13" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" t="s">
         <v>29</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" t="s">
         <v>42</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="D13" t="s">
         <v>55</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="E13" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="131.15" x14ac:dyDescent="0.4">
-      <c r="A14" s="2" t="s">
+    <row r="14" spans="1:5">
+      <c r="A14" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" t="s">
         <v>30</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" t="s">
         <v>43</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="D14" t="s">
         <v>56</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="E14" t="s">
         <v>69</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(generator): refine profiler logic with semantic transformer
- Applied semantic transformer to enhance profiling accuracy
- Adjusted profiler logic for better contextual understanding
- Improved integration with generator module to produce more coherent outputs
</commit_message>
<xml_diff>
--- a/Text2SQL_Template/output/generated_datasets/ddq_autogen_customer.xlsx
+++ b/Text2SQL_Template/output/generated_datasets/ddq_autogen_customer.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="105">
   <si>
     <t>document</t>
   </si>
@@ -31,25 +31,34 @@
     <t>metadata</t>
   </si>
   <si>
-    <t>customer | Tra cứu mã</t>
-  </si>
-  <si>
-    <t>customer | Tra cứu số mã khách hàng</t>
-  </si>
-  <si>
-    <t>customer | Tra cứu định danh khách hàng nội bộ</t>
-  </si>
-  <si>
-    <t>customer | Tra cứu mã số khách hàng</t>
-  </si>
-  <si>
-    <t>customer | Tra cứu số khách hàng chi nhánh</t>
-  </si>
-  <si>
-    <t>customer | Lọc theo loại số khách hàng</t>
-  </si>
-  <si>
-    <t>customer | Lọc theo khách hàng trạng thái</t>
+    <t>customer | Tra cứu customer information file</t>
+  </si>
+  <si>
+    <t>customer | Tra cứu id định danh khách hàng trong nội bộ</t>
+  </si>
+  <si>
+    <t>customer | Tra cứu có thể khác với cif tùy theo cấu trúc hệ thống</t>
+  </si>
+  <si>
+    <t>customer | Lọc theo họ và tên đầy đủ khách hàng</t>
+  </si>
+  <si>
+    <t>customer | Tra cứu quản lý mã cif</t>
+  </si>
+  <si>
+    <t>customer | Lọc theo khách hàng ưu tiên...</t>
+  </si>
+  <si>
+    <t>customer | Lọc theo address line</t>
+  </si>
+  <si>
+    <t>customer | Tra cứu mã chi nhánh quản lý trực tiếp khách hàng</t>
+  </si>
+  <si>
+    <t>customer | Lọc theo inactive</t>
+  </si>
+  <si>
+    <t>customer | Tra cứu ngày cấp giấy tờ định danh</t>
   </si>
   <si>
     <t>customer | Lọc thời gian theo ngày khởi tạo khách hàng trên</t>
@@ -58,37 +67,58 @@
     <t>customer | Thống kê đánh dấu khách hàng có thuộc diện mặc định thu phí hay không</t>
   </si>
   <si>
-    <t>customer | Lọc theo 1-hiệu lực</t>
+    <t>customer | Tra cứu place of issue</t>
+  </si>
+  <si>
+    <t>customer | Tra cứu trạng thái số tiền</t>
+  </si>
+  <si>
+    <t>customer | Lọc theo trạng thái</t>
   </si>
   <si>
     <t>customer | Lọc thời gian theo ngày trạng thái trạng thái</t>
   </si>
   <si>
-    <t>customer | Lọc theo trước khi thay đổi</t>
+    <t>customer | Lọc theo người thụ hưởng khách hàng trạng thái</t>
   </si>
   <si>
     <t>customer | Lọc theo trạng thái new khách hàng</t>
   </si>
   <si>
-    <t>Tìm kiếm chính xác theo mã</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác theo số mã khách hàng</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác theo định danh khách hàng nội bộ</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác theo mã số khách hàng</t>
-  </si>
-  <si>
-    <t>Tìm kiếm chính xác theo số khách hàng chi nhánh</t>
-  </si>
-  <si>
-    <t>Phân nhóm giao dịch theo loại số khách hàng</t>
-  </si>
-  <si>
-    <t>Phân nhóm giao dịch theo khách hàng trạng thái</t>
+    <t>customer | Tra cứu unique image front</t>
+  </si>
+  <si>
+    <t>customer | Tra cứu unique image back</t>
+  </si>
+  <si>
+    <t>Tìm kiếm chính xác theo customer information file</t>
+  </si>
+  <si>
+    <t>Tìm kiếm chính xác theo id định danh khách hàng trong nội bộ</t>
+  </si>
+  <si>
+    <t>Tìm kiếm chính xác theo có thể khác với cif tùy theo cấu trúc hệ thống</t>
+  </si>
+  <si>
+    <t>Phân nhóm giao dịch theo họ và tên đầy đủ khách hàng</t>
+  </si>
+  <si>
+    <t>Tìm kiếm chính xác theo quản lý mã cif</t>
+  </si>
+  <si>
+    <t>Phân nhóm giao dịch theo khách hàng ưu tiên...</t>
+  </si>
+  <si>
+    <t>Phân nhóm giao dịch theo address line</t>
+  </si>
+  <si>
+    <t>Tìm kiếm chính xác theo mã chi nhánh quản lý trực tiếp khách hàng</t>
+  </si>
+  <si>
+    <t>Phân nhóm giao dịch theo inactive</t>
+  </si>
+  <si>
+    <t>Tìm kiếm chính xác theo ngày cấp giấy tờ định danh</t>
   </si>
   <si>
     <t>Truy vấn lịch sử dựa trên cột ngày khởi tạo khách hàng trên</t>
@@ -97,186 +127,282 @@
     <t>Tính tổng giá trị đánh dấu khách hàng có thuộc diện mặc định thu phí hay không</t>
   </si>
   <si>
-    <t>Phân nhóm giao dịch theo 1-hiệu lực</t>
+    <t>Tìm kiếm chính xác theo place of issue</t>
+  </si>
+  <si>
+    <t>Tìm kiếm chính xác theo trạng thái số tiền</t>
+  </si>
+  <si>
+    <t>Phân nhóm giao dịch theo trạng thái</t>
   </si>
   <si>
     <t>Truy vấn lịch sử dựa trên cột ngày trạng thái trạng thái</t>
   </si>
   <si>
-    <t>Phân nhóm giao dịch theo trước khi thay đổi</t>
+    <t>Phân nhóm giao dịch theo người thụ hưởng khách hàng trạng thái</t>
   </si>
   <si>
     <t>Phân nhóm giao dịch theo trạng thái new khách hàng</t>
   </si>
   <si>
-    <t>Search khách hàng 591 hôm nay
-Kiểm tra lệnh 591 đang ở trạng thái nào
-Search chi tiết khách hàng số 591
-Check giao dịch 591</t>
-  </si>
-  <si>
-    <t>Search khách hàng 840 hôm nay
-Check giao dịch 840
-Kiểm tra lệnh 840 đang ở trạng thái nào
-Search chi tiết khách hàng số 840</t>
-  </si>
-  <si>
-    <t>Sao kê cho số mã khách hàng 1016000
-Danh sách giao dịch của khách hàng 1016000
-Xem lịch sử của số mã khách hàng 1016000</t>
-  </si>
-  <si>
-    <t>Các giao dịch của khách hàng 6912068
-Xem lịch sử của số mã khách hàng 6912068
-Sao kê cho số mã khách hàng 6912068</t>
-  </si>
-  <si>
-    <t>Các giao dịch của khách hàng 5492284
-Xem lịch sử của định danh khách hàng nội bộ 5492284
-Sao kê cho định danh khách hàng nội bộ 5492284</t>
-  </si>
-  <si>
-    <t>Sao kê cho định danh khách hàng nội bộ 3381737
-Xem lịch sử của định danh khách hàng nội bộ 3381737
-Danh sách giao dịch của khách hàng 3381737</t>
-  </si>
-  <si>
-    <t>Xem lịch sử của mã số khách hàng 3396081
-Sao kê cho mã số khách hàng 3396081
-Danh sách giao dịch của khách hàng 3396081</t>
-  </si>
-  <si>
-    <t>Xem lịch sử của mã số khách hàng 6288255
-Sao kê cho mã số khách hàng 6288255
-Các giao dịch của khách hàng 6288255</t>
-  </si>
-  <si>
-    <t>Xem lịch sử của số khách hàng chi nhánh TYPE_SX80
-Sao kê cho số khách hàng chi nhánh TYPE_SX80
-Những giao dịch của khách hàng TYPE_SX80</t>
-  </si>
-  <si>
-    <t>Xem lịch sử của số khách hàng chi nhánh GRP_XLE4
-Những giao dịch của khách hàng GRP_XLE4
-Sao kê cho số khách hàng chi nhánh GRP_XLE4</t>
-  </si>
-  <si>
-    <t>Hiển thị khách hàng theo loại số khách hàng hóa đơn điện
-Hiển thị những khách hàng có loại số khách hàng là hóa đơn điện</t>
-  </si>
-  <si>
-    <t>Liệt kê khách hàng theo loại số khách hàng hóa đơn nước
-Liệt kê những khách hàng có loại số khách hàng là hóa đơn nước</t>
-  </si>
-  <si>
-    <t>Những những khách hàng có khách hàng trạng thái là hết hạn
-Những khách hàng theo khách hàng trạng thái hết hạn</t>
-  </si>
-  <si>
-    <t>Kiểm tra danh sách khách hàng là lỗi
-Tra cứu danh sách khách hàng là quá giờ
-Tra cứu các khách hàng quá giờ
-khách hàng lỗi
+    <t>Tìm kiếm chính xác theo unique image front</t>
+  </si>
+  <si>
+    <t>Tìm kiếm chính xác theo unique image back</t>
+  </si>
+  <si>
+    <t>Vui lòng Liệt kê thông tin chi tiết của khách hàng có customer information file là 2041164
+Check customer information file 2041164
+Tìm kiếm khách hàng ứng với số 2041164
+Tra cứu khách hàng 2041164
+Xem chi tiết 2041164
+Thông tin về khách hàng số 2041164
+Hãy hiển thị dữ liệu bản ghi khách hàng với customer information file 2041164
+Search customer information file 2041164 là của ai?
+Liệt kê khách hàng theo customer information file 2041164</t>
+  </si>
+  <si>
+    <t>Vui lòng Search thông tin chi tiết của khách hàng có id định danh khách hàng trong nội bộ là 7658264
+Hiển thị khách hàng theo id định danh khách hàng trong nội bộ 7658264
+Xem chi tiết 7658264
+Check id định danh khách hàng trong nội bộ 7658264
+Kiểm tra khách hàng 7658264
+Tìm kiếm khách hàng ứng với số 7658264
+Hãy hiển thị dữ liệu bản ghi khách hàng với id định danh khách hàng trong nội bộ 7658264
+Thông tin về khách hàng số 7658264
+Kiểm tra id định danh khách hàng trong nội bộ 7658264 là của ai?</t>
+  </si>
+  <si>
+    <t>Check có thể khác với cif tùy theo cấu trúc hệ thống 1093818
+Xem chi tiết 1093818
+Thông tin về khách hàng số 1093818
+Search có thể khác với cif tùy theo cấu trúc hệ thống 1093818 là của ai?
+Tìm khách hàng theo có thể khác với cif tùy theo cấu trúc hệ thống 1093818
+Hãy hiển thị dữ liệu bản ghi khách hàng với có thể khác với cif tùy theo cấu trúc hệ thống 1093818
+Tìm kiếm khách hàng ứng với số 1093818
+Vui lòng Tìm thông tin chi tiết của khách hàng có có thể khác với cif tùy theo cấu trúc hệ thống là 1093818
+Hiển thị khách hàng 1093818</t>
+  </si>
+  <si>
+    <t>Trích xuất báo cáo các khách hàng thuộc loại CAT_VUEL
+Những khách hàng nào là CAT_VUEL?
+Cho xem danh sách khách hàng CAT_VUEL
+Tìm tất cả khách hàng loại CAT_VUEL
+Lọc các khách hàng đang ở trạng thái CAT_VUEL
+Danh sách CAT_VUEL
+Hãy liệt kê danh sách các khách hàng có họ và tên đầy đủ khách hàng là CAT_VUEL</t>
+  </si>
+  <si>
+    <t>Hãy hiển thị dữ liệu bản ghi khách hàng với quản lý mã cif MODE_JNWQ
+Vui lòng Tra cứu thông tin chi tiết của khách hàng có quản lý mã cif là MODE_JNWQ
+Xem chi tiết khách hàng MODE_JNWQ
+Kiểm tra khách hàng theo quản lý mã cif MODE_JNWQ
+Tìm kiếm khách hàng ứng với số MODE_JNWQ
+Tra cứu quản lý mã cif MODE_JNWQ là của ai?
+Thông tin về khách hàng số MODE_JNWQ
+Xem chi tiết MODE_JNWQ
+Check quản lý mã cif MODE_JNWQ</t>
+  </si>
+  <si>
+    <t>Những khách hàng nào là hóa đơn nước?
+Lọc các khách hàng đang ở trạng thái hóa đơn nước
+Tìm tất cả khách hàng loại hóa đơn nước
+Hãy liệt kê danh sách các khách hàng có khách hàng ưu tiên... là hóa đơn nước
+Cho xem danh sách khách hàng hóa đơn nước
+Danh sách hóa đơn nước
+Trích xuất báo cáo các khách hàng thuộc loại hóa đơn nước</t>
+  </si>
+  <si>
+    <t>Những khách hàng nào là TYPE_AVHP?
+Danh sách TYPE_AVHP
+Cho xem danh sách khách hàng TYPE_AVHP
+Hãy liệt kê danh sách các khách hàng có address line là TYPE_AVHP
+Lọc các khách hàng đang ở trạng thái TYPE_AVHP
+Trích xuất báo cáo các khách hàng thuộc loại TYPE_AVHP
+Tìm tất cả khách hàng loại TYPE_AVHP</t>
+  </si>
+  <si>
+    <t>Xem chi tiết khách hàng theo mã chi nhánh quản lý trực tiếp khách hàng hóa đơn điện
+Tìm kiếm khách hàng ứng với số hóa đơn điện
+Xem chi tiết hóa đơn điện
+Vui lòng Search thông tin chi tiết của khách hàng có mã chi nhánh quản lý trực tiếp khách hàng là hóa đơn điện
+Hãy hiển thị dữ liệu bản ghi khách hàng với mã chi nhánh quản lý trực tiếp khách hàng hóa đơn điện
+Check mã chi nhánh quản lý trực tiếp khách hàng hóa đơn điện
+Kiểm tra khách hàng hóa đơn điện
+Thông tin về khách hàng số hóa đơn điện
+Kiểm tra mã chi nhánh quản lý trực tiếp khách hàng hóa đơn điện là của ai?</t>
+  </si>
+  <si>
+    <t>Liệt kê các khách hàng hết hạn
+Những khách hàng nào là hết hạn?
+Những các khách hàng đang chờ
+khách hàng đang chờ
+Kiểm tra danh sách khách hàng là thất bại
+Hãy liệt kê danh sách các khách hàng có inactive là hết hạn
+Lọc các khách hàng đang ở trạng thái hết hạn
+Cho xem danh sách khách hàng hết hạn
+khách hàng thất bại
+Danh sách hết hạn
+Trích xuất báo cáo các khách hàng thuộc loại hết hạn
+Những danh sách khách hàng là đang chờ
+Kiểm tra các khách hàng thất bại
+Tìm tất cả khách hàng loại hết hạn
+khách hàng hết hạn
+Liệt kê danh sách khách hàng là hết hạn</t>
+  </si>
+  <si>
+    <t>Liệt kê khách hàng 2025-10-23
+Xem chi tiết 2025-10-23
+Xem chi tiết khách hàng theo ngày cấp giấy tờ định danh 2025-10-23
+Thông tin về khách hàng số 2025-10-23
+Tra cứu ngày cấp giấy tờ định danh 2025-10-23 là của ai?
+Check ngày cấp giấy tờ định danh 2025-10-23
+Vui lòng Xem chi tiết thông tin chi tiết của khách hàng có ngày cấp giấy tờ định danh là 2025-10-23
+Tìm kiếm khách hàng ứng với số 2025-10-23
+Hãy hiển thị dữ liệu bản ghi khách hàng với ngày cấp giấy tờ định danh 2025-10-23</t>
+  </si>
+  <si>
+    <t>Sao kê khách hàng theo ngày khởi tạo khách hàng trên từ ngày 2026-01-14 đến ngày 2026-02-05
+Lọc khách hàng có ngày khởi tạo khách hàng trên trong khoảng 2026-01-14 - 2026-02-05
+Xem lịch sử khách hàng dựa trên ngày khởi tạo khách hàng trên từ 2026-01-14 tới 2026-02-05</t>
+  </si>
+  <si>
+    <t>Tổng đánh dấu khách hàng có thuộc diện mặc định thu phí hay không là bao nhiêu?
+Tính tổng đánh dấu khách hàng có thuộc diện mặc định thu phí hay không
+Thống kê đánh dấu khách hàng có thuộc diện mặc định thu phí hay không hôm nay</t>
+  </si>
+  <si>
+    <t>Vui lòng Cho tôi xem thông tin chi tiết của khách hàng có place of issue là TYPE_VO25
+Hiển thị place of issue TYPE_VO25 là của ai?
+Thông tin về khách hàng số TYPE_VO25
+Cho tôi xem khách hàng TYPE_VO25
+Xem chi tiết khách hàng theo place of issue TYPE_VO25
+Check place of issue TYPE_VO25
+Hãy hiển thị dữ liệu bản ghi khách hàng với place of issue TYPE_VO25
+Tìm kiếm khách hàng ứng với số TYPE_VO25
+Xem chi tiết TYPE_VO25</t>
+  </si>
+  <si>
+    <t>Vui lòng Kiểm tra thông tin chi tiết của khách hàng có trạng thái số tiền là GRP_J0AH
+Xem chi tiết GRP_J0AH
+Tra cứu trạng thái số tiền GRP_J0AH là của ai?
+Check trạng thái số tiền GRP_J0AH
+Tìm kiếm khách hàng ứng với số GRP_J0AH
+Hiển thị khách hàng theo trạng thái số tiền GRP_J0AH
+Thông tin về khách hàng số GRP_J0AH
+Hãy hiển thị dữ liệu bản ghi khách hàng với trạng thái số tiền GRP_J0AH
+Kiểm tra khách hàng GRP_J0AH</t>
+  </si>
+  <si>
+    <t>Hiển thị danh sách khách hàng là quá giờ
+Kiểm tra các khách hàng treo
+Kiểm tra danh sách khách hàng là treo
+Liệt kê các khách hàng đã xong
 khách hàng quá giờ
-Kiểm tra các khách hàng lỗi
-khách hàng đã xong
-Search các khách hàng đã xong
-Search danh sách khách hàng là đã xong</t>
-  </si>
-  <si>
-    <t>Sao kê khách hàng theo ngày khởi tạo khách hàng trên từ ngày 2026-01-22 đến ngày 2026-02-03
-Lọc khách hàng có ngày khởi tạo khách hàng trên trong khoảng 2026-01-22 - 2026-02-03
-Xem lịch sử khách hàng dựa trên ngày khởi tạo khách hàng trên từ 2026-01-22 tới 2026-02-03
-Kiểm tra các khách hàng với ngày khởi tạo khách hàng trên là ngày 2026-01-22</t>
-  </si>
-  <si>
-    <t>Sao kê khách hàng theo ngày khởi tạo khách hàng trên từ ngày 2026-01-12 đến ngày 2026-02-03
-Lọc khách hàng có ngày khởi tạo khách hàng trên trong khoảng 2026-01-12 - 2026-02-03
-Xem lịch sử khách hàng dựa trên ngày khởi tạo khách hàng trên từ 2026-01-12 tới 2026-02-03
-Kiểm tra các khách hàng với ngày khởi tạo khách hàng trên là ngày 2026-01-12</t>
-  </si>
-  <si>
-    <t>Tổng đánh dấu khách hàng có thuộc diện mặc định thu phí hay không là bao nhiêu?
-Tính tổng đánh dấu khách hàng có thuộc diện mặc định thu phí hay không của các giao dịch thành công
-Thống kê đánh dấu khách hàng có thuộc diện mặc định thu phí hay không hôm nay</t>
-  </si>
-  <si>
-    <t>Những khách hàng theo 1-hiệu lực đã xong
-Những những khách hàng có 1-hiệu lực là đã xong</t>
-  </si>
-  <si>
-    <t>Kiểm tra danh sách khách hàng là hết hạn
-Kiểm tra các khách hàng hết hạn
-Search danh sách khách hàng là bị treo
-Danh sách các khách hàng hoàn tất
-Search các khách hàng bị treo
+khách hàng treo
+Lọc các khách hàng đang ở trạng thái hết hạn
+Những khách hàng nào là hết hạn?
+Cho xem danh sách khách hàng hết hạn
+Danh sách hết hạn
+Hiển thị các khách hàng quá giờ
+Trích xuất báo cáo các khách hàng thuộc loại hết hạn
+Hãy liệt kê danh sách các khách hàng có trạng thái là hết hạn
+Tìm tất cả khách hàng loại hết hạn
+Liệt kê danh sách khách hàng là đã xong
+khách hàng đã xong</t>
+  </si>
+  <si>
+    <t>Sao kê khách hàng theo ngày trạng thái trạng thái từ ngày 2025-12-14 đến ngày 2026-02-05
+Lọc khách hàng có ngày trạng thái trạng thái trong khoảng 2025-12-14 - 2026-02-05
+Xem lịch sử khách hàng dựa trên ngày trạng thái trạng thái từ 2025-12-14 tới 2026-02-05</t>
+  </si>
+  <si>
+    <t>khách hàng thành công
+Liệt kê danh sách khách hàng là treo
+Trích xuất báo cáo các khách hàng thuộc loại bị treo
+Lọc các khách hàng đang ở trạng thái bị treo
+Liệt kê các khách hàng treo
+Danh sách các khách hàng hết hạn
+Hãy liệt kê danh sách các khách hàng có người thụ hưởng khách hàng trạng thái là bị treo
+Liệt kê danh sách khách hàng là thành công
+Liệt kê các khách hàng thành công
+Những khách hàng nào là bị treo?
+Danh sách bị treo
+Tìm tất cả khách hàng loại bị treo
+Danh sách danh sách khách hàng là hết hạn
 khách hàng hết hạn
-khách hàng bị treo
-Danh sách danh sách khách hàng là hoàn tất
-khách hàng hoàn tất</t>
-  </si>
-  <si>
-    <t>Sao kê khách hàng theo ngày trạng thái trạng thái từ ngày 2025-12-23 đến ngày 2026-02-03
-Lọc khách hàng có ngày trạng thái trạng thái trong khoảng 2025-12-23 - 2026-02-03
-Xem lịch sử khách hàng dựa trên ngày trạng thái trạng thái từ 2025-12-23 tới 2026-02-03
-Kiểm tra các khách hàng với ngày trạng thái trạng thái là ngày 2025-12-23</t>
-  </si>
-  <si>
-    <t>Sao kê khách hàng theo ngày trạng thái trạng thái từ ngày 2025-12-10 đến ngày 2026-02-03
-Lọc khách hàng có ngày trạng thái trạng thái trong khoảng 2025-12-10 - 2026-02-03
-Xem lịch sử khách hàng dựa trên ngày trạng thái trạng thái từ 2025-12-10 tới 2026-02-03
-Kiểm tra các khách hàng với ngày trạng thái trạng thái là ngày 2025-12-10</t>
-  </si>
-  <si>
-    <t>Lọc các những khách hàng có trước khi thay đổi là quá giờ
-Lọc các khách hàng theo trước khi thay đổi quá giờ</t>
-  </si>
-  <si>
-    <t>Các các khách hàng hết hạn
-khách hàng thành công
-khách hàng xử lý
-Các danh sách khách hàng là hết hạn
-Tìm danh sách khách hàng là xử lý
+Cho xem danh sách khách hàng bị treo
+khách hàng treo</t>
+  </si>
+  <si>
+    <t>Những khách hàng nào là xử lý?
+khách hàng hoàn tất
+Lọc các khách hàng đang ở trạng thái xử lý
+Hãy liệt kê danh sách các khách hàng có trạng thái new khách hàng là xử lý
+Cho xem danh sách khách hàng xử lý
+Những các khách hàng thất bại
+khách hàng thất bại
+Search các khách hàng hoàn tất
+Tìm danh sách khách hàng là hết hạn
+Tìm các khách hàng hết hạn
+Search danh sách khách hàng là hoàn tất
+Tìm tất cả khách hàng loại xử lý
+Những danh sách khách hàng là thất bại
+Danh sách xử lý
 khách hàng hết hạn
-Tra cứu danh sách khách hàng là thành công
-Tìm các khách hàng xử lý
-Tra cứu các khách hàng thành công</t>
-  </si>
-  <si>
-    <t>Cho tôi xem những khách hàng có trạng thái new khách hàng là thành công
-Cho tôi xem khách hàng theo trạng thái new khách hàng thành công</t>
-  </si>
-  <si>
-    <t>Cho tôi xem các khách hàng xử lý
-Tìm các khách hàng bị treo
-khách hàng thành công
-Cho tôi xem danh sách khách hàng là xử lý
-Xem chi tiết danh sách khách hàng là thành công
-khách hàng xử lý
-khách hàng bị treo
-Xem chi tiết các khách hàng thành công
-Tìm danh sách khách hàng là bị treo</t>
-  </si>
-  <si>
-    <t>mã, id tự tăng là khóa chính bản ghi này, số, bản ghi này, primary key</t>
-  </si>
-  <si>
-    <t>số mã khách hàng, mã khách hàng, customer information file, số cif, số khách hàng, mã định danh khách hàng, số số khách hàng, số cif mã định danh duy nhất khách hàng ngân hàng</t>
-  </si>
-  <si>
-    <t>định danh khách hàng nội bộ, id định danh khách hàng trong nội bộ, số khách hàng, mã khách hàng</t>
-  </si>
-  <si>
-    <t>mã số khách hàng, số khách hàng, có thể khác với cif tùy theo cấu trúc hệ thống</t>
-  </si>
-  <si>
-    <t>số khách hàng chi nhánh, khách hàng chi nhánh, quản lý mã cif này, chi nhánh nơi mở, mã khách hàng chi nhánh, chi nhánh nơi mở/quản lý mã cif này</t>
-  </si>
-  <si>
-    <t>loại số khách hàng, loại mã khách hàng, loại cif, khách hàng ưu tiên..., loại khách hàng, doanh nghiệp, cá nhân</t>
-  </si>
-  <si>
-    <t>khách hàng trạng thái, trạng thái khách hàng, trạng thái hiện khách hàng, inactive, closed..., active</t>
+Trích xuất báo cáo các khách hàng thuộc loại xử lý</t>
+  </si>
+  <si>
+    <t>Liệt kê unique image front TYPE_KQ7P là của ai?
+Thông tin về khách hàng số TYPE_KQ7P
+Check unique image front TYPE_KQ7P
+Tìm kiếm khách hàng ứng với số TYPE_KQ7P
+Vui lòng Xem chi tiết thông tin chi tiết của khách hàng có unique image front là TYPE_KQ7P
+Search khách hàng TYPE_KQ7P
+Hãy hiển thị dữ liệu bản ghi khách hàng với unique image front TYPE_KQ7P
+Xem chi tiết TYPE_KQ7P
+Hiển thị khách hàng theo unique image front TYPE_KQ7P</t>
+  </si>
+  <si>
+    <t>Tìm kiếm khách hàng ứng với số GRP_2H2S
+Thông tin về khách hàng số GRP_2H2S
+Check unique image back GRP_2H2S
+Hãy hiển thị dữ liệu bản ghi khách hàng với unique image back GRP_2H2S
+Xem chi tiết khách hàng GRP_2H2S
+Liệt kê unique image back GRP_2H2S là của ai?
+Xem chi tiết GRP_2H2S
+Vui lòng Search thông tin chi tiết của khách hàng có unique image back là GRP_2H2S
+Hiển thị khách hàng theo unique image back GRP_2H2S</t>
+  </si>
+  <si>
+    <t>customer information file, số mã khách hàng, mã định danh khách hàng, số cif mã định danh duy nhất khách hàng ngân hàng, số số khách hàng, số cif, mã khách hàng, số khách hàng</t>
+  </si>
+  <si>
+    <t>id định danh khách hàng trong nội bộ, số khách hàng, mã khách hàng</t>
+  </si>
+  <si>
+    <t>có thể khác với cif tùy theo cấu trúc hệ thống, số khách hàng, mã số khách hàng</t>
+  </si>
+  <si>
+    <t>họ và tên đầy đủ khách hàng, tên khách hàng</t>
+  </si>
+  <si>
+    <t>quản lý mã cif, chi nhánh nơi mở/quản lý mã cif này, khách hàng chi nhánh, chi nhánh nơi mở, mã khách hàng chi nhánh, số khách hàng chi nhánh</t>
+  </si>
+  <si>
+    <t>khách hàng ưu tiên..., cá nhân, loại cif, doanh nghiệp, loại số khách hàng, loại khách hàng, loại mã khách hàng</t>
+  </si>
+  <si>
+    <t>address line, dòng địa chỉ chi tiết, tên đường, số tài khoản trạng thái, số nhà, dòng địa chỉ</t>
+  </si>
+  <si>
+    <t>mã chi nhánh quản lý trực tiếp khách hàng, số chi nhánh, mã chi nhánh</t>
+  </si>
+  <si>
+    <t>inactive, trạng thái hiện khách hàng, khách hàng trạng thái, trạng thái khách hàng, active, closed...</t>
+  </si>
+  <si>
+    <t>ngày cấp giấy tờ định danh, cmnd/cccd/hộ chiếu, ngày trạng thái trạng thái, ngày of issue</t>
   </si>
   <si>
     <t>thời gian, lịch sử, ngày khởi tạo khách hàng trên</t>
@@ -285,19 +411,28 @@
     <t>tổng, thống kê, theo đánh dấu khách hàng có thuộc diện mặc định thu phí hay không</t>
   </si>
   <si>
-    <t>1-hiệu lực, trạng thái bản ghi, trạng thái, 0-hết hiệu lực</t>
+    <t>place of issue, nội dung trạng thái trạng thái, nơi cấp giấy tờ định danh, ca tp. hà nội</t>
+  </si>
+  <si>
+    <t>trạng thái số tiền, giá trị đặc trưng định danh duy nhất khách hàng, unique value</t>
+  </si>
+  <si>
+    <t>trạng thái, 0-hết hiệu lực, trạng thái bản ghi, 1-hiệu lực</t>
   </si>
   <si>
     <t>thời gian, lịch sử, ngày trạng thái trạng thái</t>
   </si>
   <si>
-    <t>trước khi thay đổi, người thụ hưởng khách hàng trạng thái, trạng thái cũ khách hàng, trạng thái old khách hàng</t>
+    <t>người thụ hưởng khách hàng trạng thái, trạng thái old khách hàng, trước khi thay đổi, trạng thái cũ khách hàng</t>
   </si>
   <si>
     <t>trạng thái new khách hàng, nội dung khách hàng trạng thái, sau khi cập nhật, trạng thái mới khách hàng</t>
   </si>
   <si>
-    <t>{"raw_text": "SELECT * FROM customer WHERE id = '{{id}}'"}</t>
+    <t>unique image front, cmnd/cccd, đường dẫn ảnh mặt trước giấy tờ định danh, trạng thái nội dung trạng thái</t>
+  </si>
+  <si>
+    <t>unique image back, đường dẫn ảnh mặt sau giấy tờ định danh, trạng thái nội dung trạng thái</t>
   </si>
   <si>
     <t>{"raw_text": "SELECT * FROM customer WHERE cif_no = '{{cif_no}}'"}</t>
@@ -309,21 +444,39 @@
     <t>{"raw_text": "SELECT * FROM customer WHERE customer_no = '{{customer_no}}'"}</t>
   </si>
   <si>
+    <t>{"raw_text": "SELECT * FROM customer WHERE customer_name = '{{customer_name}}' AND new_customer_status = 'SUCCESS'"}</t>
+  </si>
+  <si>
     <t>{"raw_text": "SELECT * FROM customer WHERE cif_branch = '{{cif_branch}}'"}</t>
   </si>
   <si>
     <t>{"raw_text": "SELECT * FROM customer WHERE cif_type = '{{cif_type}}' AND new_customer_status = 'SUCCESS'"}</t>
   </si>
   <si>
+    <t>{"raw_text": "SELECT * FROM customer WHERE address_line = '{{address_line}}' AND new_customer_status = 'SUCCESS'"}</t>
+  </si>
+  <si>
+    <t>{"raw_text": "SELECT * FROM customer WHERE branch_code = '{{branch_code}}'"}</t>
+  </si>
+  <si>
     <t>{"raw_text": "SELECT * FROM customer WHERE customer_status = '{{customer_status}}'"}</t>
   </si>
   <si>
+    <t>{"raw_text": "SELECT * FROM customer WHERE date_of_issue = '{{date_of_issue}}'"}</t>
+  </si>
+  <si>
     <t>{"raw_text": "SELECT * FROM customer WHERE init_date BETWEEN '{{start_date}}' AND '{{end_date}}' ORDER BY init_date DESC"}</t>
   </si>
   <si>
     <t>{"raw_text": "SELECT SUM(is_fee_default) FROM customer WHERE new_customer_status = 'SUCCESS'"}</t>
   </si>
   <si>
+    <t>{"raw_text": "SELECT * FROM customer WHERE place_of_issue = '{{place_of_issue}}'"}</t>
+  </si>
+  <si>
+    <t>{"raw_text": "SELECT * FROM customer WHERE unique_value = '{{unique_value}}'"}</t>
+  </si>
+  <si>
     <t>{"raw_text": "SELECT * FROM customer WHERE status = '{{status}}'"}</t>
   </si>
   <si>
@@ -334,6 +487,12 @@
   </si>
   <si>
     <t>{"raw_text": "SELECT * FROM customer WHERE new_customer_status = '{{new_customer_status}}'"}</t>
+  </si>
+  <si>
+    <t>{"raw_text": "SELECT * FROM customer WHERE unique_image_front = '{{unique_image_front}}'"}</t>
+  </si>
+  <si>
+    <t>{"raw_text": "SELECT * FROM customer WHERE unique_image_back = '{{unique_image_back}}'"}</t>
   </si>
 </sst>
 </file>
@@ -691,7 +850,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -716,441 +875,339 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="C2" t="s">
-        <v>31</v>
+        <v>45</v>
       </c>
       <c r="D2" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E2" t="s">
-        <v>69</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="C3" t="s">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="D3" t="s">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="E3" t="s">
-        <v>69</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="C4" t="s">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="D4" t="s">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="E4" t="s">
-        <v>70</v>
+        <v>87</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="D5" t="s">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="E5" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="C6" t="s">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="D6" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="E6" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
+        <v>50</v>
       </c>
       <c r="D7" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="E7" t="s">
-        <v>71</v>
+        <v>90</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="C8" t="s">
-        <v>37</v>
+        <v>51</v>
       </c>
       <c r="D8" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="E8" t="s">
-        <v>72</v>
+        <v>91</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B9" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="C9" t="s">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="D9" t="s">
-        <v>59</v>
+        <v>72</v>
       </c>
       <c r="E9" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B10" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="C10" t="s">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="D10" t="s">
-        <v>60</v>
+        <v>73</v>
       </c>
       <c r="E10" t="s">
-        <v>73</v>
+        <v>93</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B11" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="C11" t="s">
-        <v>40</v>
+        <v>54</v>
       </c>
       <c r="D11" t="s">
-        <v>60</v>
+        <v>74</v>
       </c>
       <c r="E11" t="s">
-        <v>73</v>
+        <v>94</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B12" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="C12" t="s">
-        <v>41</v>
+        <v>55</v>
       </c>
       <c r="D12" t="s">
-        <v>61</v>
+        <v>75</v>
       </c>
       <c r="E12" t="s">
-        <v>74</v>
+        <v>95</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="B13" t="s">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="C13" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="D13" t="s">
-        <v>61</v>
+        <v>76</v>
       </c>
       <c r="E13" t="s">
-        <v>74</v>
+        <v>96</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="B14" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="C14" t="s">
-        <v>43</v>
+        <v>57</v>
       </c>
       <c r="D14" t="s">
-        <v>62</v>
+        <v>77</v>
       </c>
       <c r="E14" t="s">
-        <v>75</v>
+        <v>97</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="B15" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="C15" t="s">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="D15" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="E15" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="B16" t="s">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="C16" t="s">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="D16" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="E16" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="B17" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="C17" t="s">
-        <v>46</v>
+        <v>60</v>
       </c>
       <c r="D17" t="s">
-        <v>63</v>
+        <v>80</v>
       </c>
       <c r="E17" t="s">
-        <v>76</v>
+        <v>100</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="B18" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="C18" t="s">
-        <v>47</v>
+        <v>61</v>
       </c>
       <c r="D18" t="s">
-        <v>64</v>
+        <v>81</v>
       </c>
       <c r="E18" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="B19" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="C19" t="s">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="D19" t="s">
-        <v>64</v>
+        <v>82</v>
       </c>
       <c r="E19" t="s">
-        <v>77</v>
+        <v>102</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="B20" t="s">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="C20" t="s">
-        <v>48</v>
+        <v>63</v>
       </c>
       <c r="D20" t="s">
-        <v>65</v>
+        <v>83</v>
       </c>
       <c r="E20" t="s">
-        <v>78</v>
+        <v>103</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="B21" t="s">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="C21" t="s">
-        <v>49</v>
+        <v>64</v>
       </c>
       <c r="D21" t="s">
-        <v>65</v>
+        <v>84</v>
       </c>
       <c r="E21" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5">
-      <c r="A22" t="s">
-        <v>15</v>
-      </c>
-      <c r="B22" t="s">
-        <v>28</v>
-      </c>
-      <c r="C22" t="s">
-        <v>50</v>
-      </c>
-      <c r="D22" t="s">
-        <v>66</v>
-      </c>
-      <c r="E22" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5">
-      <c r="A23" t="s">
-        <v>15</v>
-      </c>
-      <c r="B23" t="s">
-        <v>28</v>
-      </c>
-      <c r="C23" t="s">
-        <v>51</v>
-      </c>
-      <c r="D23" t="s">
-        <v>66</v>
-      </c>
-      <c r="E23" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5">
-      <c r="A24" t="s">
-        <v>16</v>
-      </c>
-      <c r="B24" t="s">
-        <v>29</v>
-      </c>
-      <c r="C24" t="s">
-        <v>52</v>
-      </c>
-      <c r="D24" t="s">
-        <v>67</v>
-      </c>
-      <c r="E24" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5">
-      <c r="A25" t="s">
-        <v>16</v>
-      </c>
-      <c r="B25" t="s">
-        <v>29</v>
-      </c>
-      <c r="C25" t="s">
-        <v>53</v>
-      </c>
-      <c r="D25" t="s">
-        <v>67</v>
-      </c>
-      <c r="E25" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5">
-      <c r="A26" t="s">
-        <v>17</v>
-      </c>
-      <c r="B26" t="s">
-        <v>30</v>
-      </c>
-      <c r="C26" t="s">
-        <v>54</v>
-      </c>
-      <c r="D26" t="s">
-        <v>68</v>
-      </c>
-      <c r="E26" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5">
-      <c r="A27" t="s">
-        <v>17</v>
-      </c>
-      <c r="B27" t="s">
-        <v>30</v>
-      </c>
-      <c r="C27" t="s">
-        <v>55</v>
-      </c>
-      <c r="D27" t="s">
-        <v>68</v>
-      </c>
-      <c r="E27" t="s">
-        <v>81</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>

</xml_diff>